<commit_message>
Updating code and unit tests to use 'orf_n_terminus_index' when refering to the starting position of the ORF and associated protein. Expected results have also been updated to account of the way in which ORF on negative strands are recorded.
</commit_message>
<xml_diff>
--- a/orfaqs/tests/python/modules/orfaqsproteindiscovery/data/discovered-proteins/expected-results/expected-discovered-proteins.xlsx
+++ b/orfaqs/tests/python/modules/orfaqsproteindiscovery/data/discovered-proteins/expected-results/expected-discovered-proteins.xlsx
@@ -1,34 +1,100 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cashby/dev/projects/orfaqs/orfaqs/tests/python/modules/orfaqsproteindiscovery/data/discovered-proteins/expected-results/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6EE0EA0-786E-7444-A792-5777F1DE0E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>source_uid</t>
+  </si>
+  <si>
+    <t>strand_type</t>
+  </si>
+  <si>
+    <t>reading_frame</t>
+  </si>
+  <si>
+    <t>protein</t>
+  </si>
+  <si>
+    <t>protein_length</t>
+  </si>
+  <si>
+    <t>unknown_reference</t>
+  </si>
+  <si>
+    <t>positive_strand</t>
+  </si>
+  <si>
+    <t>MNEICSAHPTI</t>
+  </si>
+  <si>
+    <t>MKYAPLIPPSN</t>
+  </si>
+  <si>
+    <t>MLRSSHHLTS</t>
+  </si>
+  <si>
+    <t>negative_strand</t>
+  </si>
+  <si>
+    <t>MVG</t>
+  </si>
+  <si>
+    <t>orf_n_terminus_index</t>
+  </si>
+  <si>
+    <t>genomic_sequence</t>
+  </si>
+  <si>
+    <t>TCAGCTAGTTAGATGGTGGGATGAGCGGAGCATTAA</t>
+  </si>
+  <si>
+    <t>GCTAGTTAGATGGTGGGATGAGCGGAGCATATTTAA</t>
+  </si>
+  <si>
+    <t>TAGATGGTGGGATGAGCGGAGCATATTTCATAA</t>
+  </si>
+  <si>
+    <t>ATGGTGGGATAATAA</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +113,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,164 +415,141 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_uid</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>strand_type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>reading_frame</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>dna_sequence_position</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>protein</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>protein_length</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>unknown_reference</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>positive_strand</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>MNEICSAHPTI</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2">
         <v>11</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>unknown_reference</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>positive_strand</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>4</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>MKYAPLIPPSN</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3">
         <v>11</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>unknown_reference</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>positive_strand</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4">
         <v>3</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>10</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>MLRSSHHLTS</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
         <v>10</v>
       </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>unknown_reference</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>negative_strand</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>MVG</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
+      <c r="E5">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Bugfix/accuracy and nomenclature (#26)
* Changing references of 'genomic_sequence' to 'orf_n_terminus'. This terminology is more precise and reflective of what is being captured.

* [BUGFIX] The genomic sequence should include the nucleotides associated with the stop codon. The protein should not. Now all genomic sequences include the stop codon.

* Refactoring: arranging the order of columns in the ORFaqProteinQeury related databases.

* Updating code and unit tests to use 'orf_n_terminus_index' when refering to the starting position of the ORF and associated protein. Expected results have also been updated to account of the way in which ORF on negative strands are recorded.

* Adding the ability to index triplets from the tail end of a GenomicSequence object. Adding test conditions to validate recorded genomic sequences include the stop codon, while the recorded protein does not.
</commit_message>
<xml_diff>
--- a/orfaqs/tests/python/modules/orfaqsproteindiscovery/data/discovered-proteins/expected-results/expected-discovered-proteins.xlsx
+++ b/orfaqs/tests/python/modules/orfaqsproteindiscovery/data/discovered-proteins/expected-results/expected-discovered-proteins.xlsx
@@ -1,34 +1,100 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cashby/dev/projects/orfaqs/orfaqs/tests/python/modules/orfaqsproteindiscovery/data/discovered-proteins/expected-results/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6EE0EA0-786E-7444-A792-5777F1DE0E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>source_uid</t>
+  </si>
+  <si>
+    <t>strand_type</t>
+  </si>
+  <si>
+    <t>reading_frame</t>
+  </si>
+  <si>
+    <t>protein</t>
+  </si>
+  <si>
+    <t>protein_length</t>
+  </si>
+  <si>
+    <t>unknown_reference</t>
+  </si>
+  <si>
+    <t>positive_strand</t>
+  </si>
+  <si>
+    <t>MNEICSAHPTI</t>
+  </si>
+  <si>
+    <t>MKYAPLIPPSN</t>
+  </si>
+  <si>
+    <t>MLRSSHHLTS</t>
+  </si>
+  <si>
+    <t>negative_strand</t>
+  </si>
+  <si>
+    <t>MVG</t>
+  </si>
+  <si>
+    <t>orf_n_terminus_index</t>
+  </si>
+  <si>
+    <t>genomic_sequence</t>
+  </si>
+  <si>
+    <t>TCAGCTAGTTAGATGGTGGGATGAGCGGAGCATTAA</t>
+  </si>
+  <si>
+    <t>GCTAGTTAGATGGTGGGATGAGCGGAGCATATTTAA</t>
+  </si>
+  <si>
+    <t>TAGATGGTGGGATGAGCGGAGCATATTTCATAA</t>
+  </si>
+  <si>
+    <t>ATGGTGGGATAATAA</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +113,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,164 +415,141 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>source_uid</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>strand_type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>reading_frame</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>dna_sequence_position</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>protein</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>protein_length</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>unknown_reference</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>positive_strand</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>MNEICSAHPTI</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2">
         <v>11</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>unknown_reference</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>positive_strand</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>4</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>MKYAPLIPPSN</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3">
         <v>11</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>unknown_reference</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>positive_strand</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4">
         <v>3</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>10</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>MLRSSHHLTS</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
         <v>10</v>
       </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>unknown_reference</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>negative_strand</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>MVG</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
+      <c r="E5">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5">
         <v>3</v>
       </c>
     </row>

</xml_diff>